<commit_message>
Update source files, Remove columns from export, reorder columns, rename high-risk -> co-occuring conditions
</commit_message>
<xml_diff>
--- a/characteristics_tables/Influenza_Study_Characteristics.xlsx
+++ b/characteristics_tables/Influenza_Study_Characteristics.xlsx
@@ -1818,7 +1818,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B13">
         <v>1259</v>
@@ -1936,7 +1936,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B14">
         <v>1322</v>
@@ -2054,7 +2054,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B15">
         <v>1344</v>
@@ -2307,7 +2307,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B17">
         <v>1418</v>
@@ -2425,7 +2425,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B18">
         <v>1420</v>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B19">
         <v>1429</v>
@@ -2666,7 +2666,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B20">
         <v>1441</v>
@@ -2789,7 +2789,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B21">
         <v>1506</v>
@@ -2921,7 +2921,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B22">
         <v>1572</v>
@@ -3044,7 +3044,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B23">
         <v>1647</v>
@@ -3172,7 +3172,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B24">
         <v>1664</v>
@@ -3290,7 +3290,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B25">
         <v>1905</v>
@@ -3419,7 +3419,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B26">
         <v>1920</v>
@@ -3547,7 +3547,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B27">
         <v>1924</v>
@@ -3675,7 +3675,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B28">
         <v>1960</v>
@@ -3788,7 +3788,7 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B29">
         <v>1969</v>
@@ -3901,7 +3901,7 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B30">
         <v>1970</v>
@@ -4260,7 +4260,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B33">
         <v>2150</v>
@@ -4383,7 +4383,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B34">
         <v>21829</v>
@@ -4511,7 +4511,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B35">
         <v>2420</v>
@@ -4629,7 +4629,7 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B36">
         <v>2680</v>
@@ -4860,7 +4860,7 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B38">
         <v>3183</v>
@@ -5232,7 +5232,7 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B41">
         <v>32935</v>
@@ -5601,7 +5601,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B44">
         <v>3947</v>
@@ -5729,7 +5729,7 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B45">
         <v>4110</v>
@@ -6114,7 +6114,7 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B48">
         <v>4748</v>
@@ -6360,7 +6360,7 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B50">
         <v>5196</v>
@@ -6601,7 +6601,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B52">
         <v>5246</v>
@@ -6724,7 +6724,7 @@
     </row>
     <row r="53">
       <c r="A53">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B53">
         <v>5422</v>
@@ -6852,7 +6852,7 @@
     </row>
     <row r="54">
       <c r="A54">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B54">
         <v>5445</v>
@@ -6986,7 +6986,7 @@
     </row>
     <row r="55">
       <c r="A55">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B55">
         <v>5751</v>
@@ -7115,7 +7115,7 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B56">
         <v>5803</v>
@@ -7241,7 +7241,7 @@
     </row>
     <row r="57">
       <c r="A57">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B57">
         <v>5810</v>
@@ -7364,7 +7364,7 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B58">
         <v>5814</v>
@@ -11259,7 +11259,7 @@
     </row>
     <row r="74">
       <c r="A74">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B74">
         <v>1259</v>
@@ -11282,7 +11282,7 @@
     </row>
     <row r="75">
       <c r="A75">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B75">
         <v>1322</v>
@@ -11305,7 +11305,7 @@
     </row>
     <row r="76">
       <c r="A76">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B76">
         <v>1322</v>
@@ -11328,7 +11328,7 @@
     </row>
     <row r="77">
       <c r="A77">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B77">
         <v>1322</v>
@@ -11351,7 +11351,7 @@
     </row>
     <row r="78">
       <c r="A78">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B78">
         <v>1344</v>
@@ -11374,7 +11374,7 @@
     </row>
     <row r="79">
       <c r="A79">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B79">
         <v>1344</v>
@@ -11397,7 +11397,7 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B80">
         <v>1344</v>
@@ -11420,7 +11420,7 @@
     </row>
     <row r="81">
       <c r="A81">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B81">
         <v>1418</v>
@@ -11443,7 +11443,7 @@
     </row>
     <row r="82">
       <c r="A82">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B82">
         <v>1420</v>
@@ -11466,7 +11466,7 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B83">
         <v>1429</v>
@@ -11489,7 +11489,7 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B84">
         <v>1429</v>
@@ -11512,7 +11512,7 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B85">
         <v>1429</v>
@@ -11535,7 +11535,7 @@
     </row>
     <row r="86">
       <c r="A86">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B86">
         <v>1429</v>
@@ -11558,7 +11558,7 @@
     </row>
     <row r="87">
       <c r="A87">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B87">
         <v>1441</v>
@@ -11581,7 +11581,7 @@
     </row>
     <row r="88">
       <c r="A88">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B88">
         <v>1506</v>
@@ -11604,7 +11604,7 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B89">
         <v>1572</v>
@@ -11627,7 +11627,7 @@
     </row>
     <row r="90">
       <c r="A90">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B90">
         <v>1572</v>
@@ -11650,7 +11650,7 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B91">
         <v>1572</v>
@@ -11673,7 +11673,7 @@
     </row>
     <row r="92">
       <c r="A92">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B92">
         <v>1647</v>
@@ -11696,7 +11696,7 @@
     </row>
     <row r="93">
       <c r="A93">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B93">
         <v>1647</v>
@@ -11719,7 +11719,7 @@
     </row>
     <row r="94">
       <c r="A94">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B94">
         <v>1664</v>
@@ -11742,7 +11742,7 @@
     </row>
     <row r="95">
       <c r="A95">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B95">
         <v>1905</v>
@@ -11765,7 +11765,7 @@
     </row>
     <row r="96">
       <c r="A96">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B96">
         <v>1920</v>
@@ -11788,7 +11788,7 @@
     </row>
     <row r="97">
       <c r="A97">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B97">
         <v>1920</v>
@@ -11811,7 +11811,7 @@
     </row>
     <row r="98">
       <c r="A98">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B98">
         <v>1924</v>
@@ -11834,7 +11834,7 @@
     </row>
     <row r="99">
       <c r="A99">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B99">
         <v>1960</v>
@@ -11857,7 +11857,7 @@
     </row>
     <row r="100">
       <c r="A100">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B100">
         <v>1969</v>
@@ -11880,7 +11880,7 @@
     </row>
     <row r="101">
       <c r="A101">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B101">
         <v>1969</v>
@@ -11903,7 +11903,7 @@
     </row>
     <row r="102">
       <c r="A102">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B102">
         <v>1969</v>
@@ -11926,7 +11926,7 @@
     </row>
     <row r="103">
       <c r="A103">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B103">
         <v>1970</v>
@@ -11949,7 +11949,7 @@
     </row>
     <row r="104">
       <c r="A104">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B104">
         <v>2150</v>
@@ -11972,7 +11972,7 @@
     </row>
     <row r="105">
       <c r="A105">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B105">
         <v>2150</v>
@@ -11995,7 +11995,7 @@
     </row>
     <row r="106">
       <c r="A106">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B106">
         <v>2420</v>
@@ -12018,7 +12018,7 @@
     </row>
     <row r="107">
       <c r="A107">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B107">
         <v>2680</v>
@@ -12041,7 +12041,7 @@
     </row>
     <row r="108">
       <c r="A108">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B108">
         <v>2680</v>
@@ -12064,7 +12064,7 @@
     </row>
     <row r="109">
       <c r="A109">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B109">
         <v>3183</v>
@@ -12087,7 +12087,7 @@
     </row>
     <row r="110">
       <c r="A110">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B110">
         <v>3947</v>
@@ -12110,7 +12110,7 @@
     </row>
     <row r="111">
       <c r="A111">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B111">
         <v>3947</v>
@@ -12133,7 +12133,7 @@
     </row>
     <row r="112">
       <c r="A112">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B112">
         <v>4110</v>
@@ -12156,7 +12156,7 @@
     </row>
     <row r="113">
       <c r="A113">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B113">
         <v>4110</v>
@@ -12179,7 +12179,7 @@
     </row>
     <row r="114">
       <c r="A114">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B114">
         <v>4110</v>
@@ -12202,7 +12202,7 @@
     </row>
     <row r="115">
       <c r="A115">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B115">
         <v>4748</v>
@@ -12225,7 +12225,7 @@
     </row>
     <row r="116">
       <c r="A116">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B116">
         <v>4748</v>
@@ -12248,7 +12248,7 @@
     </row>
     <row r="117">
       <c r="A117">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B117">
         <v>4748</v>
@@ -12271,7 +12271,7 @@
     </row>
     <row r="118">
       <c r="A118">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B118">
         <v>5196</v>
@@ -12294,7 +12294,7 @@
     </row>
     <row r="119">
       <c r="A119">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B119">
         <v>5246</v>
@@ -12317,7 +12317,7 @@
     </row>
     <row r="120">
       <c r="A120">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B120">
         <v>5246</v>
@@ -12340,7 +12340,7 @@
     </row>
     <row r="121">
       <c r="A121">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B121">
         <v>5422</v>
@@ -12363,7 +12363,7 @@
     </row>
     <row r="122">
       <c r="A122">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B122">
         <v>5445</v>
@@ -12386,7 +12386,7 @@
     </row>
     <row r="123">
       <c r="A123">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B123">
         <v>5751</v>
@@ -12409,7 +12409,7 @@
     </row>
     <row r="124">
       <c r="A124">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B124">
         <v>5751</v>
@@ -12432,7 +12432,7 @@
     </row>
     <row r="125">
       <c r="A125">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B125">
         <v>5803</v>
@@ -12455,7 +12455,7 @@
     </row>
     <row r="126">
       <c r="A126">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B126">
         <v>5803</v>
@@ -12478,7 +12478,7 @@
     </row>
     <row r="127">
       <c r="A127">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B127">
         <v>5803</v>
@@ -12501,7 +12501,7 @@
     </row>
     <row r="128">
       <c r="A128">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B128">
         <v>5810</v>
@@ -12524,7 +12524,7 @@
     </row>
     <row r="129">
       <c r="A129">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B129">
         <v>5810</v>
@@ -12547,7 +12547,7 @@
     </row>
     <row r="130">
       <c r="A130">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B130">
         <v>5814</v>
@@ -12570,7 +12570,7 @@
     </row>
     <row r="131">
       <c r="A131">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B131">
         <v>5814</v>
@@ -12593,7 +12593,7 @@
     </row>
     <row r="132">
       <c r="A132">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B132">
         <v>21829</v>
@@ -12616,7 +12616,7 @@
     </row>
     <row r="133">
       <c r="A133">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B133">
         <v>21829</v>
@@ -12639,7 +12639,7 @@
     </row>
     <row r="134">
       <c r="A134">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B134">
         <v>32935</v>
@@ -12662,7 +12662,7 @@
     </row>
     <row r="135">
       <c r="A135">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B135">
         <v>32935</v>
@@ -12685,7 +12685,7 @@
     </row>
     <row r="136">
       <c r="A136">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B136">
         <v>32935</v>
@@ -12708,7 +12708,7 @@
     </row>
     <row r="137">
       <c r="A137">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B137">
         <v>32935</v>
@@ -12731,7 +12731,7 @@
     </row>
     <row r="138">
       <c r="A138">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B138">
         <v>32935</v>
@@ -12754,7 +12754,7 @@
     </row>
     <row r="139">
       <c r="A139">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B139">
         <v>32935</v>
@@ -12777,7 +12777,7 @@
     </row>
     <row r="140">
       <c r="A140">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B140">
         <v>32935</v>
@@ -12992,7 +12992,7 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B12">
         <v>1259</v>
@@ -13008,7 +13008,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B13">
         <v>1322</v>
@@ -13024,7 +13024,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B14">
         <v>1344</v>
@@ -13056,7 +13056,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16">
         <v>1418</v>
@@ -13072,7 +13072,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17">
         <v>1420</v>
@@ -13088,7 +13088,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B18">
         <v>1429</v>
@@ -13104,7 +13104,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B19">
         <v>1506</v>
@@ -13120,7 +13120,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B20">
         <v>1572</v>
@@ -13136,7 +13136,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B21">
         <v>1647</v>
@@ -13152,7 +13152,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B22">
         <v>1664</v>
@@ -13168,7 +13168,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B23">
         <v>1905</v>
@@ -13184,7 +13184,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B24">
         <v>1920</v>
@@ -13200,7 +13200,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B25">
         <v>1924</v>
@@ -13216,7 +13216,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B26">
         <v>1960</v>
@@ -13232,7 +13232,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B27">
         <v>1969</v>
@@ -13248,7 +13248,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B28">
         <v>1970</v>
@@ -13296,7 +13296,7 @@
     </row>
     <row r="31">
       <c r="A31">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31">
         <v>2150</v>
@@ -13312,7 +13312,7 @@
     </row>
     <row r="32">
       <c r="A32">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B32">
         <v>21829</v>
@@ -13328,7 +13328,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B33">
         <v>2680</v>
@@ -13360,7 +13360,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B35">
         <v>3183</v>
@@ -13408,7 +13408,7 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B38">
         <v>32935</v>
@@ -13440,7 +13440,7 @@
     </row>
     <row r="40">
       <c r="A40">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B40">
         <v>3947</v>
@@ -13456,7 +13456,7 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B41">
         <v>4110</v>
@@ -13504,7 +13504,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B44">
         <v>4748</v>
@@ -13536,7 +13536,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B46">
         <v>5196</v>
@@ -13568,7 +13568,7 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B48">
         <v>5246</v>
@@ -13584,7 +13584,7 @@
     </row>
     <row r="49">
       <c r="A49">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B49">
         <v>5422</v>
@@ -13600,7 +13600,7 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B50">
         <v>5445</v>
@@ -13616,7 +13616,7 @@
     </row>
     <row r="51">
       <c r="A51">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B51">
         <v>5751</v>
@@ -13632,7 +13632,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B52">
         <v>5803</v>
@@ -13648,7 +13648,7 @@
     </row>
     <row r="53">
       <c r="A53">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B53">
         <v>5810</v>
@@ -13664,7 +13664,7 @@
     </row>
     <row r="54">
       <c r="A54">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B54">
         <v>5814</v>
@@ -14508,7 +14508,7 @@
     </row>
     <row r="32">
       <c r="A32">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B32">
         <v>1259</v>
@@ -14526,7 +14526,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33">
         <v>1259</v>
@@ -14544,7 +14544,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B34">
         <v>1259</v>
@@ -14562,7 +14562,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B35">
         <v>1322</v>
@@ -14580,7 +14580,7 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B36">
         <v>1322</v>
@@ -14598,7 +14598,7 @@
     </row>
     <row r="37">
       <c r="A37">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B37">
         <v>1344</v>
@@ -14616,7 +14616,7 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B38">
         <v>1344</v>
@@ -14706,7 +14706,7 @@
     </row>
     <row r="43">
       <c r="A43">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B43">
         <v>1418</v>
@@ -14724,7 +14724,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B44">
         <v>1420</v>
@@ -14742,7 +14742,7 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B45">
         <v>1420</v>
@@ -14760,7 +14760,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B46">
         <v>1429</v>
@@ -14778,7 +14778,7 @@
     </row>
     <row r="47">
       <c r="A47">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B47">
         <v>1429</v>
@@ -14796,7 +14796,7 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B48">
         <v>1429</v>
@@ -14814,7 +14814,7 @@
     </row>
     <row r="49">
       <c r="A49">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B49">
         <v>1441</v>
@@ -14832,7 +14832,7 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B50">
         <v>1441</v>
@@ -14850,7 +14850,7 @@
     </row>
     <row r="51">
       <c r="A51">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B51">
         <v>1441</v>
@@ -14868,7 +14868,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B52">
         <v>1441</v>
@@ -14886,7 +14886,7 @@
     </row>
     <row r="53">
       <c r="A53">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B53">
         <v>1506</v>
@@ -14904,7 +14904,7 @@
     </row>
     <row r="54">
       <c r="A54">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B54">
         <v>1506</v>
@@ -14922,7 +14922,7 @@
     </row>
     <row r="55">
       <c r="A55">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B55">
         <v>1572</v>
@@ -14940,7 +14940,7 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B56">
         <v>1572</v>
@@ -14958,7 +14958,7 @@
     </row>
     <row r="57">
       <c r="A57">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B57">
         <v>1647</v>
@@ -14976,7 +14976,7 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B58">
         <v>1647</v>
@@ -14994,7 +14994,7 @@
     </row>
     <row r="59">
       <c r="A59">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B59">
         <v>1664</v>
@@ -15012,7 +15012,7 @@
     </row>
     <row r="60">
       <c r="A60">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B60">
         <v>1664</v>
@@ -15030,7 +15030,7 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B61">
         <v>1664</v>
@@ -15048,7 +15048,7 @@
     </row>
     <row r="62">
       <c r="A62">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B62">
         <v>1664</v>
@@ -15066,7 +15066,7 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B63">
         <v>1905</v>
@@ -15084,7 +15084,7 @@
     </row>
     <row r="64">
       <c r="A64">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B64">
         <v>1905</v>
@@ -15102,7 +15102,7 @@
     </row>
     <row r="65">
       <c r="A65">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B65">
         <v>1920</v>
@@ -15120,7 +15120,7 @@
     </row>
     <row r="66">
       <c r="A66">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B66">
         <v>1920</v>
@@ -15138,7 +15138,7 @@
     </row>
     <row r="67">
       <c r="A67">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B67">
         <v>1924</v>
@@ -15156,7 +15156,7 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B68">
         <v>1960</v>
@@ -15174,7 +15174,7 @@
     </row>
     <row r="69">
       <c r="A69">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B69">
         <v>1960</v>
@@ -15192,7 +15192,7 @@
     </row>
     <row r="70">
       <c r="A70">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B70">
         <v>1960</v>
@@ -15210,7 +15210,7 @@
     </row>
     <row r="71">
       <c r="A71">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B71">
         <v>1960</v>
@@ -15228,7 +15228,7 @@
     </row>
     <row r="72">
       <c r="A72">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B72">
         <v>1969</v>
@@ -15246,7 +15246,7 @@
     </row>
     <row r="73">
       <c r="A73">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B73">
         <v>1969</v>
@@ -15264,7 +15264,7 @@
     </row>
     <row r="74">
       <c r="A74">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B74">
         <v>1970</v>
@@ -15282,7 +15282,7 @@
     </row>
     <row r="75">
       <c r="A75">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B75">
         <v>1970</v>
@@ -15354,7 +15354,7 @@
     </row>
     <row r="79">
       <c r="A79">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B79">
         <v>2150</v>
@@ -15372,7 +15372,7 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B80">
         <v>2150</v>
@@ -15390,7 +15390,7 @@
     </row>
     <row r="81">
       <c r="A81">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B81">
         <v>21829</v>
@@ -15408,7 +15408,7 @@
     </row>
     <row r="82">
       <c r="A82">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B82">
         <v>21829</v>
@@ -15426,7 +15426,7 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B83">
         <v>2420</v>
@@ -15444,7 +15444,7 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B84">
         <v>2420</v>
@@ -15462,7 +15462,7 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B85">
         <v>2420</v>
@@ -15480,7 +15480,7 @@
     </row>
     <row r="86">
       <c r="A86">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B86">
         <v>2420</v>
@@ -15498,7 +15498,7 @@
     </row>
     <row r="87">
       <c r="A87">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B87">
         <v>2680</v>
@@ -15534,7 +15534,7 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B89">
         <v>3183</v>
@@ -15552,7 +15552,7 @@
     </row>
     <row r="90">
       <c r="A90">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B90">
         <v>3183</v>
@@ -15570,7 +15570,7 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B91">
         <v>3183</v>
@@ -15588,7 +15588,7 @@
     </row>
     <row r="92">
       <c r="A92">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B92">
         <v>3183</v>
@@ -15678,7 +15678,7 @@
     </row>
     <row r="97">
       <c r="A97">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B97">
         <v>32935</v>
@@ -15696,7 +15696,7 @@
     </row>
     <row r="98">
       <c r="A98">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B98">
         <v>32935</v>
@@ -15750,7 +15750,7 @@
     </row>
     <row r="101">
       <c r="A101">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B101">
         <v>3947</v>
@@ -15768,7 +15768,7 @@
     </row>
     <row r="102">
       <c r="A102">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B102">
         <v>3947</v>
@@ -15786,7 +15786,7 @@
     </row>
     <row r="103">
       <c r="A103">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B103">
         <v>3947</v>
@@ -15804,7 +15804,7 @@
     </row>
     <row r="104">
       <c r="A104">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B104">
         <v>3947</v>
@@ -15822,7 +15822,7 @@
     </row>
     <row r="105">
       <c r="A105">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B105">
         <v>4110</v>
@@ -15912,7 +15912,7 @@
     </row>
     <row r="110">
       <c r="A110">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B110">
         <v>4748</v>
@@ -15930,7 +15930,7 @@
     </row>
     <row r="111">
       <c r="A111">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B111">
         <v>4748</v>
@@ -15984,7 +15984,7 @@
     </row>
     <row r="114">
       <c r="A114">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B114">
         <v>5196</v>
@@ -16038,7 +16038,7 @@
     </row>
     <row r="117">
       <c r="A117">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B117">
         <v>5246</v>
@@ -16056,7 +16056,7 @@
     </row>
     <row r="118">
       <c r="A118">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B118">
         <v>5246</v>
@@ -16074,7 +16074,7 @@
     </row>
     <row r="119">
       <c r="A119">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B119">
         <v>5422</v>
@@ -16092,7 +16092,7 @@
     </row>
     <row r="120">
       <c r="A120">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B120">
         <v>5445</v>
@@ -16110,7 +16110,7 @@
     </row>
     <row r="121">
       <c r="A121">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B121">
         <v>5445</v>
@@ -16128,7 +16128,7 @@
     </row>
     <row r="122">
       <c r="A122">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B122">
         <v>5751</v>
@@ -16146,7 +16146,7 @@
     </row>
     <row r="123">
       <c r="A123">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B123">
         <v>5751</v>
@@ -16164,7 +16164,7 @@
     </row>
     <row r="124">
       <c r="A124">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B124">
         <v>5751</v>
@@ -16182,7 +16182,7 @@
     </row>
     <row r="125">
       <c r="A125">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B125">
         <v>5751</v>
@@ -16200,7 +16200,7 @@
     </row>
     <row r="126">
       <c r="A126">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B126">
         <v>5803</v>
@@ -16218,7 +16218,7 @@
     </row>
     <row r="127">
       <c r="A127">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B127">
         <v>5803</v>
@@ -16236,7 +16236,7 @@
     </row>
     <row r="128">
       <c r="A128">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B128">
         <v>5810</v>
@@ -16254,7 +16254,7 @@
     </row>
     <row r="129">
       <c r="A129">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B129">
         <v>5814</v>
@@ -17150,7 +17150,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B15">
         <v>1259</v>
@@ -17168,7 +17168,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B16">
         <v>1259</v>
@@ -17186,7 +17186,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B17">
         <v>1322</v>
@@ -17204,7 +17204,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B18">
         <v>1344</v>
@@ -17240,7 +17240,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B20">
         <v>1418</v>
@@ -17258,7 +17258,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B21">
         <v>1420</v>
@@ -17276,7 +17276,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B22">
         <v>1429</v>
@@ -17294,7 +17294,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B23">
         <v>1441</v>
@@ -17312,7 +17312,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B24">
         <v>1506</v>
@@ -17330,7 +17330,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B25">
         <v>1572</v>
@@ -17348,7 +17348,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B26">
         <v>1647</v>
@@ -17366,7 +17366,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27">
         <v>1664</v>
@@ -17384,7 +17384,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B28">
         <v>1905</v>
@@ -17402,7 +17402,7 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B29">
         <v>1905</v>
@@ -17420,7 +17420,7 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B30">
         <v>1920</v>
@@ -17438,7 +17438,7 @@
     </row>
     <row r="31">
       <c r="A31">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B31">
         <v>1924</v>
@@ -17456,7 +17456,7 @@
     </row>
     <row r="32">
       <c r="A32">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B32">
         <v>1924</v>
@@ -17474,7 +17474,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B33">
         <v>1960</v>
@@ -17492,7 +17492,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B34">
         <v>1969</v>
@@ -17510,7 +17510,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B35">
         <v>1970</v>
@@ -17528,7 +17528,7 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B36">
         <v>1970</v>
@@ -17546,7 +17546,7 @@
     </row>
     <row r="37">
       <c r="A37">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B37">
         <v>1970</v>
@@ -17600,7 +17600,7 @@
     </row>
     <row r="40">
       <c r="A40">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B40">
         <v>2150</v>
@@ -17618,7 +17618,7 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B41">
         <v>2150</v>
@@ -17636,7 +17636,7 @@
     </row>
     <row r="42">
       <c r="A42">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B42">
         <v>2150</v>
@@ -17654,7 +17654,7 @@
     </row>
     <row r="43">
       <c r="A43">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B43">
         <v>21829</v>
@@ -17672,7 +17672,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B44">
         <v>21829</v>
@@ -17690,7 +17690,7 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B45">
         <v>2420</v>
@@ -17708,7 +17708,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B46">
         <v>2680</v>
@@ -17744,7 +17744,7 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B48">
         <v>3183</v>
@@ -17798,7 +17798,7 @@
     </row>
     <row r="51">
       <c r="A51">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B51">
         <v>32935</v>
@@ -17816,7 +17816,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B52">
         <v>32935</v>
@@ -17888,7 +17888,7 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B56">
         <v>3947</v>
@@ -17906,7 +17906,7 @@
     </row>
     <row r="57">
       <c r="A57">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B57">
         <v>4110</v>
@@ -17924,7 +17924,7 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B58">
         <v>4110</v>
@@ -17978,7 +17978,7 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B61">
         <v>4748</v>
@@ -18014,7 +18014,7 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B63">
         <v>5196</v>
@@ -18050,7 +18050,7 @@
     </row>
     <row r="65">
       <c r="A65">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B65">
         <v>5246</v>
@@ -18068,7 +18068,7 @@
     </row>
     <row r="66">
       <c r="A66">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B66">
         <v>5422</v>
@@ -18086,7 +18086,7 @@
     </row>
     <row r="67">
       <c r="A67">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B67">
         <v>5445</v>
@@ -18104,7 +18104,7 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B68">
         <v>5751</v>
@@ -18122,7 +18122,7 @@
     </row>
     <row r="69">
       <c r="A69">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B69">
         <v>5803</v>
@@ -18140,7 +18140,7 @@
     </row>
     <row r="70">
       <c r="A70">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B70">
         <v>5810</v>
@@ -18158,7 +18158,7 @@
     </row>
     <row r="71">
       <c r="A71">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B71">
         <v>5814</v>
@@ -23103,7 +23103,7 @@
     </row>
     <row r="207">
       <c r="A207">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B207">
         <v>1259</v>
@@ -23126,7 +23126,7 @@
     </row>
     <row r="208">
       <c r="A208">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B208">
         <v>1259</v>
@@ -23149,7 +23149,7 @@
     </row>
     <row r="209">
       <c r="A209">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B209">
         <v>1259</v>
@@ -23172,7 +23172,7 @@
     </row>
     <row r="210">
       <c r="A210">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B210">
         <v>1259</v>
@@ -23195,7 +23195,7 @@
     </row>
     <row r="211">
       <c r="A211">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B211">
         <v>1259</v>
@@ -23218,7 +23218,7 @@
     </row>
     <row r="212">
       <c r="A212">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B212">
         <v>1259</v>
@@ -23241,7 +23241,7 @@
     </row>
     <row r="213">
       <c r="A213">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B213">
         <v>1259</v>
@@ -23264,7 +23264,7 @@
     </row>
     <row r="214">
       <c r="A214">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B214">
         <v>1259</v>
@@ -23287,7 +23287,7 @@
     </row>
     <row r="215">
       <c r="A215">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B215">
         <v>1259</v>
@@ -23310,7 +23310,7 @@
     </row>
     <row r="216">
       <c r="A216">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B216">
         <v>1259</v>
@@ -23333,7 +23333,7 @@
     </row>
     <row r="217">
       <c r="A217">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B217">
         <v>1259</v>
@@ -23356,7 +23356,7 @@
     </row>
     <row r="218">
       <c r="A218">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B218">
         <v>1259</v>
@@ -23379,7 +23379,7 @@
     </row>
     <row r="219">
       <c r="A219">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B219">
         <v>1259</v>
@@ -23402,7 +23402,7 @@
     </row>
     <row r="220">
       <c r="A220">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B220">
         <v>1259</v>
@@ -23425,7 +23425,7 @@
     </row>
     <row r="221">
       <c r="A221">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B221">
         <v>1259</v>
@@ -23448,7 +23448,7 @@
     </row>
     <row r="222">
       <c r="A222">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B222">
         <v>1259</v>
@@ -23471,7 +23471,7 @@
     </row>
     <row r="223">
       <c r="A223">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B223">
         <v>1322</v>
@@ -23494,7 +23494,7 @@
     </row>
     <row r="224">
       <c r="A224">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B224">
         <v>1322</v>
@@ -23517,7 +23517,7 @@
     </row>
     <row r="225">
       <c r="A225">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B225">
         <v>1322</v>
@@ -23540,7 +23540,7 @@
     </row>
     <row r="226">
       <c r="A226">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B226">
         <v>1322</v>
@@ -23563,7 +23563,7 @@
     </row>
     <row r="227">
       <c r="A227">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B227">
         <v>1322</v>
@@ -23586,7 +23586,7 @@
     </row>
     <row r="228">
       <c r="A228">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B228">
         <v>1322</v>
@@ -23609,7 +23609,7 @@
     </row>
     <row r="229">
       <c r="A229">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B229">
         <v>1418</v>
@@ -23632,7 +23632,7 @@
     </row>
     <row r="230">
       <c r="A230">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B230">
         <v>1418</v>
@@ -23655,7 +23655,7 @@
     </row>
     <row r="231">
       <c r="A231">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B231">
         <v>1420</v>
@@ -23678,7 +23678,7 @@
     </row>
     <row r="232">
       <c r="A232">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B232">
         <v>1420</v>
@@ -23701,7 +23701,7 @@
     </row>
     <row r="233">
       <c r="A233">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B233">
         <v>1420</v>
@@ -23724,7 +23724,7 @@
     </row>
     <row r="234">
       <c r="A234">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B234">
         <v>1420</v>
@@ -23747,7 +23747,7 @@
     </row>
     <row r="235">
       <c r="A235">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B235">
         <v>1420</v>
@@ -23770,7 +23770,7 @@
     </row>
     <row r="236">
       <c r="A236">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B236">
         <v>1420</v>
@@ -23793,7 +23793,7 @@
     </row>
     <row r="237">
       <c r="A237">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B237">
         <v>1429</v>
@@ -23816,7 +23816,7 @@
     </row>
     <row r="238">
       <c r="A238">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B238">
         <v>1429</v>
@@ -23839,7 +23839,7 @@
     </row>
     <row r="239">
       <c r="A239">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B239">
         <v>1429</v>
@@ -23862,7 +23862,7 @@
     </row>
     <row r="240">
       <c r="A240">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B240">
         <v>1429</v>
@@ -23885,7 +23885,7 @@
     </row>
     <row r="241">
       <c r="A241">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B241">
         <v>1429</v>
@@ -23908,7 +23908,7 @@
     </row>
     <row r="242">
       <c r="A242">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B242">
         <v>1429</v>
@@ -23931,7 +23931,7 @@
     </row>
     <row r="243">
       <c r="A243">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B243">
         <v>1429</v>
@@ -23954,7 +23954,7 @@
     </row>
     <row r="244">
       <c r="A244">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B244">
         <v>1429</v>
@@ -23977,7 +23977,7 @@
     </row>
     <row r="245">
       <c r="A245">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B245">
         <v>1429</v>
@@ -24000,7 +24000,7 @@
     </row>
     <row r="246">
       <c r="A246">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B246">
         <v>1429</v>
@@ -24023,7 +24023,7 @@
     </row>
     <row r="247">
       <c r="A247">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B247">
         <v>1429</v>
@@ -24046,7 +24046,7 @@
     </row>
     <row r="248">
       <c r="A248">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B248">
         <v>1429</v>
@@ -24069,7 +24069,7 @@
     </row>
     <row r="249">
       <c r="A249">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B249">
         <v>1429</v>
@@ -24092,7 +24092,7 @@
     </row>
     <row r="250">
       <c r="A250">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B250">
         <v>1441</v>
@@ -24115,7 +24115,7 @@
     </row>
     <row r="251">
       <c r="A251">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B251">
         <v>1441</v>
@@ -24138,7 +24138,7 @@
     </row>
     <row r="252">
       <c r="A252">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B252">
         <v>1441</v>
@@ -24161,7 +24161,7 @@
     </row>
     <row r="253">
       <c r="A253">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B253">
         <v>1441</v>
@@ -24184,7 +24184,7 @@
     </row>
     <row r="254">
       <c r="A254">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B254">
         <v>1572</v>
@@ -24207,7 +24207,7 @@
     </row>
     <row r="255">
       <c r="A255">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B255">
         <v>1572</v>
@@ -24230,7 +24230,7 @@
     </row>
     <row r="256">
       <c r="A256">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B256">
         <v>1572</v>
@@ -24253,7 +24253,7 @@
     </row>
     <row r="257">
       <c r="A257">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B257">
         <v>1647</v>
@@ -24276,7 +24276,7 @@
     </row>
     <row r="258">
       <c r="A258">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B258">
         <v>1647</v>
@@ -24299,7 +24299,7 @@
     </row>
     <row r="259">
       <c r="A259">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B259">
         <v>1647</v>
@@ -24322,7 +24322,7 @@
     </row>
     <row r="260">
       <c r="A260">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B260">
         <v>1647</v>
@@ -24345,7 +24345,7 @@
     </row>
     <row r="261">
       <c r="A261">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B261">
         <v>1647</v>
@@ -24368,7 +24368,7 @@
     </row>
     <row r="262">
       <c r="A262">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B262">
         <v>1664</v>
@@ -24391,7 +24391,7 @@
     </row>
     <row r="263">
       <c r="A263">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B263">
         <v>1664</v>
@@ -24414,7 +24414,7 @@
     </row>
     <row r="264">
       <c r="A264">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B264">
         <v>1664</v>
@@ -24437,7 +24437,7 @@
     </row>
     <row r="265">
       <c r="A265">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B265">
         <v>1664</v>
@@ -24460,7 +24460,7 @@
     </row>
     <row r="266">
       <c r="A266">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B266">
         <v>1905</v>
@@ -24483,7 +24483,7 @@
     </row>
     <row r="267">
       <c r="A267">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B267">
         <v>1920</v>
@@ -24506,7 +24506,7 @@
     </row>
     <row r="268">
       <c r="A268">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B268">
         <v>1920</v>
@@ -24529,7 +24529,7 @@
     </row>
     <row r="269">
       <c r="A269">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B269">
         <v>1920</v>
@@ -24552,7 +24552,7 @@
     </row>
     <row r="270">
       <c r="A270">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B270">
         <v>1920</v>
@@ -24575,7 +24575,7 @@
     </row>
     <row r="271">
       <c r="A271">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B271">
         <v>1920</v>
@@ -24598,7 +24598,7 @@
     </row>
     <row r="272">
       <c r="A272">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B272">
         <v>1920</v>
@@ -24621,7 +24621,7 @@
     </row>
     <row r="273">
       <c r="A273">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B273">
         <v>1920</v>
@@ -24644,7 +24644,7 @@
     </row>
     <row r="274">
       <c r="A274">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B274">
         <v>1920</v>
@@ -24667,7 +24667,7 @@
     </row>
     <row r="275">
       <c r="A275">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B275">
         <v>1920</v>
@@ -24690,7 +24690,7 @@
     </row>
     <row r="276">
       <c r="A276">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B276">
         <v>1920</v>
@@ -24713,7 +24713,7 @@
     </row>
     <row r="277">
       <c r="A277">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B277">
         <v>1920</v>
@@ -24736,7 +24736,7 @@
     </row>
     <row r="278">
       <c r="A278">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B278">
         <v>1920</v>
@@ -24759,7 +24759,7 @@
     </row>
     <row r="279">
       <c r="A279">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B279">
         <v>1920</v>
@@ -24782,7 +24782,7 @@
     </row>
     <row r="280">
       <c r="A280">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B280">
         <v>1920</v>
@@ -24805,7 +24805,7 @@
     </row>
     <row r="281">
       <c r="A281">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B281">
         <v>1920</v>
@@ -24828,7 +24828,7 @@
     </row>
     <row r="282">
       <c r="A282">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B282">
         <v>1920</v>
@@ -24851,7 +24851,7 @@
     </row>
     <row r="283">
       <c r="A283">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B283">
         <v>1920</v>
@@ -24874,7 +24874,7 @@
     </row>
     <row r="284">
       <c r="A284">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B284">
         <v>1920</v>
@@ -24897,7 +24897,7 @@
     </row>
     <row r="285">
       <c r="A285">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B285">
         <v>1920</v>
@@ -24920,7 +24920,7 @@
     </row>
     <row r="286">
       <c r="A286">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B286">
         <v>1924</v>
@@ -24943,7 +24943,7 @@
     </row>
     <row r="287">
       <c r="A287">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B287">
         <v>1924</v>
@@ -24966,7 +24966,7 @@
     </row>
     <row r="288">
       <c r="A288">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B288">
         <v>1924</v>
@@ -24989,7 +24989,7 @@
     </row>
     <row r="289">
       <c r="A289">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B289">
         <v>1924</v>
@@ -25012,7 +25012,7 @@
     </row>
     <row r="290">
       <c r="A290">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B290">
         <v>1924</v>
@@ -25035,7 +25035,7 @@
     </row>
     <row r="291">
       <c r="A291">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B291">
         <v>1924</v>
@@ -25058,7 +25058,7 @@
     </row>
     <row r="292">
       <c r="A292">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B292">
         <v>1924</v>
@@ -25081,7 +25081,7 @@
     </row>
     <row r="293">
       <c r="A293">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B293">
         <v>1924</v>
@@ -25104,7 +25104,7 @@
     </row>
     <row r="294">
       <c r="A294">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B294">
         <v>1960</v>
@@ -25127,7 +25127,7 @@
     </row>
     <row r="295">
       <c r="A295">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B295">
         <v>1969</v>
@@ -25150,7 +25150,7 @@
     </row>
     <row r="296">
       <c r="A296">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B296">
         <v>1969</v>
@@ -25173,7 +25173,7 @@
     </row>
     <row r="297">
       <c r="A297">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B297">
         <v>1969</v>
@@ -25196,7 +25196,7 @@
     </row>
     <row r="298">
       <c r="A298">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B298">
         <v>1970</v>
@@ -25219,7 +25219,7 @@
     </row>
     <row r="299">
       <c r="A299">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B299">
         <v>1970</v>
@@ -25242,7 +25242,7 @@
     </row>
     <row r="300">
       <c r="A300">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B300">
         <v>1970</v>
@@ -25265,7 +25265,7 @@
     </row>
     <row r="301">
       <c r="A301">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B301">
         <v>2150</v>
@@ -25288,7 +25288,7 @@
     </row>
     <row r="302">
       <c r="A302">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B302">
         <v>2150</v>
@@ -25311,7 +25311,7 @@
     </row>
     <row r="303">
       <c r="A303">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B303">
         <v>2150</v>
@@ -25334,7 +25334,7 @@
     </row>
     <row r="304">
       <c r="A304">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B304">
         <v>2150</v>
@@ -25357,7 +25357,7 @@
     </row>
     <row r="305">
       <c r="A305">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B305">
         <v>2150</v>
@@ -25380,7 +25380,7 @@
     </row>
     <row r="306">
       <c r="A306">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B306">
         <v>2150</v>
@@ -25403,7 +25403,7 @@
     </row>
     <row r="307">
       <c r="A307">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B307">
         <v>2150</v>
@@ -25426,7 +25426,7 @@
     </row>
     <row r="308">
       <c r="A308">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B308">
         <v>2150</v>
@@ -25449,7 +25449,7 @@
     </row>
     <row r="309">
       <c r="A309">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B309">
         <v>2150</v>
@@ -25472,7 +25472,7 @@
     </row>
     <row r="310">
       <c r="A310">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B310">
         <v>2150</v>
@@ -25495,7 +25495,7 @@
     </row>
     <row r="311">
       <c r="A311">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B311">
         <v>2150</v>
@@ -25518,7 +25518,7 @@
     </row>
     <row r="312">
       <c r="A312">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B312">
         <v>2150</v>
@@ -25541,7 +25541,7 @@
     </row>
     <row r="313">
       <c r="A313">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B313">
         <v>2420</v>
@@ -25564,7 +25564,7 @@
     </row>
     <row r="314">
       <c r="A314">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B314">
         <v>2420</v>
@@ -25587,7 +25587,7 @@
     </row>
     <row r="315">
       <c r="A315">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B315">
         <v>2420</v>
@@ -25610,7 +25610,7 @@
     </row>
     <row r="316">
       <c r="A316">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B316">
         <v>2420</v>
@@ -25633,7 +25633,7 @@
     </row>
     <row r="317">
       <c r="A317">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B317">
         <v>2420</v>
@@ -25656,7 +25656,7 @@
     </row>
     <row r="318">
       <c r="A318">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B318">
         <v>2420</v>
@@ -25679,7 +25679,7 @@
     </row>
     <row r="319">
       <c r="A319">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B319">
         <v>2420</v>
@@ -25702,7 +25702,7 @@
     </row>
     <row r="320">
       <c r="A320">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B320">
         <v>2420</v>
@@ -25725,7 +25725,7 @@
     </row>
     <row r="321">
       <c r="A321">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B321">
         <v>2420</v>
@@ -25748,7 +25748,7 @@
     </row>
     <row r="322">
       <c r="A322">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B322">
         <v>2420</v>
@@ -25771,7 +25771,7 @@
     </row>
     <row r="323">
       <c r="A323">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B323">
         <v>2420</v>
@@ -25794,7 +25794,7 @@
     </row>
     <row r="324">
       <c r="A324">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B324">
         <v>2420</v>
@@ -25817,7 +25817,7 @@
     </row>
     <row r="325">
       <c r="A325">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B325">
         <v>2420</v>
@@ -25840,7 +25840,7 @@
     </row>
     <row r="326">
       <c r="A326">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B326">
         <v>2680</v>
@@ -25863,7 +25863,7 @@
     </row>
     <row r="327">
       <c r="A327">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B327">
         <v>2680</v>
@@ -25886,7 +25886,7 @@
     </row>
     <row r="328">
       <c r="A328">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B328">
         <v>4110</v>
@@ -25909,7 +25909,7 @@
     </row>
     <row r="329">
       <c r="A329">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B329">
         <v>4110</v>
@@ -25932,7 +25932,7 @@
     </row>
     <row r="330">
       <c r="A330">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B330">
         <v>4110</v>
@@ -25955,7 +25955,7 @@
     </row>
     <row r="331">
       <c r="A331">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B331">
         <v>4110</v>
@@ -25978,7 +25978,7 @@
     </row>
     <row r="332">
       <c r="A332">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B332">
         <v>4748</v>
@@ -26001,7 +26001,7 @@
     </row>
     <row r="333">
       <c r="A333">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B333">
         <v>4748</v>
@@ -26024,7 +26024,7 @@
     </row>
     <row r="334">
       <c r="A334">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B334">
         <v>4748</v>
@@ -26047,7 +26047,7 @@
     </row>
     <row r="335">
       <c r="A335">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B335">
         <v>4748</v>
@@ -26070,7 +26070,7 @@
     </row>
     <row r="336">
       <c r="A336">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B336">
         <v>4748</v>
@@ -26093,7 +26093,7 @@
     </row>
     <row r="337">
       <c r="A337">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B337">
         <v>4748</v>
@@ -26116,7 +26116,7 @@
     </row>
     <row r="338">
       <c r="A338">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B338">
         <v>4748</v>
@@ -26139,7 +26139,7 @@
     </row>
     <row r="339">
       <c r="A339">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B339">
         <v>4748</v>
@@ -26162,7 +26162,7 @@
     </row>
     <row r="340">
       <c r="A340">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B340">
         <v>4748</v>
@@ -26185,7 +26185,7 @@
     </row>
     <row r="341">
       <c r="A341">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B341">
         <v>5196</v>
@@ -26208,7 +26208,7 @@
     </row>
     <row r="342">
       <c r="A342">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B342">
         <v>5246</v>
@@ -26226,7 +26226,7 @@
     </row>
     <row r="343">
       <c r="A343">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B343">
         <v>5246</v>
@@ -26244,7 +26244,7 @@
     </row>
     <row r="344">
       <c r="A344">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B344">
         <v>5246</v>
@@ -26262,7 +26262,7 @@
     </row>
     <row r="345">
       <c r="A345">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B345">
         <v>5246</v>
@@ -26280,7 +26280,7 @@
     </row>
     <row r="346">
       <c r="A346">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B346">
         <v>5422</v>
@@ -26303,7 +26303,7 @@
     </row>
     <row r="347">
       <c r="A347">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B347">
         <v>5803</v>
@@ -26326,7 +26326,7 @@
     </row>
     <row r="348">
       <c r="A348">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B348">
         <v>5803</v>
@@ -26349,7 +26349,7 @@
     </row>
     <row r="349">
       <c r="A349">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B349">
         <v>5803</v>
@@ -26372,7 +26372,7 @@
     </row>
     <row r="350">
       <c r="A350">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B350">
         <v>5803</v>
@@ -26395,7 +26395,7 @@
     </row>
     <row r="351">
       <c r="A351">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B351">
         <v>5810</v>
@@ -26418,7 +26418,7 @@
     </row>
     <row r="352">
       <c r="A352">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B352">
         <v>5810</v>
@@ -26441,7 +26441,7 @@
     </row>
     <row r="353">
       <c r="A353">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B353">
         <v>5810</v>
@@ -26464,7 +26464,7 @@
     </row>
     <row r="354">
       <c r="A354">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B354">
         <v>5810</v>
@@ -26487,7 +26487,7 @@
     </row>
     <row r="355">
       <c r="A355">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B355">
         <v>5810</v>
@@ -26510,7 +26510,7 @@
     </row>
     <row r="356">
       <c r="A356">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B356">
         <v>5810</v>
@@ -26533,7 +26533,7 @@
     </row>
     <row r="357">
       <c r="A357">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B357">
         <v>5810</v>
@@ -26556,7 +26556,7 @@
     </row>
     <row r="358">
       <c r="A358">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B358">
         <v>5810</v>
@@ -26579,7 +26579,7 @@
     </row>
     <row r="359">
       <c r="A359">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B359">
         <v>5814</v>
@@ -26602,7 +26602,7 @@
     </row>
     <row r="360">
       <c r="A360">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B360">
         <v>5814</v>
@@ -26625,7 +26625,7 @@
     </row>
     <row r="361">
       <c r="A361">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B361">
         <v>5814</v>
@@ -26648,7 +26648,7 @@
     </row>
     <row r="362">
       <c r="A362">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B362">
         <v>5814</v>
@@ -26671,7 +26671,7 @@
     </row>
     <row r="363">
       <c r="A363">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B363">
         <v>32935</v>
@@ -26689,7 +26689,7 @@
     </row>
     <row r="364">
       <c r="A364">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B364">
         <v>32935</v>
@@ -26707,7 +26707,7 @@
     </row>
     <row r="365">
       <c r="A365">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B365">
         <v>32935</v>
@@ -26725,7 +26725,7 @@
     </row>
     <row r="366">
       <c r="A366">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B366">
         <v>32935</v>
@@ -26743,7 +26743,7 @@
     </row>
     <row r="367">
       <c r="A367">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B367">
         <v>32935</v>
@@ -26761,7 +26761,7 @@
     </row>
     <row r="368">
       <c r="A368">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B368">
         <v>32935</v>
@@ -26779,7 +26779,7 @@
     </row>
     <row r="369">
       <c r="A369">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B369">
         <v>32935</v>
@@ -26797,7 +26797,7 @@
     </row>
     <row r="370">
       <c r="A370">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B370">
         <v>32935</v>
@@ -26815,7 +26815,7 @@
     </row>
     <row r="371">
       <c r="A371">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B371">
         <v>32935</v>
@@ -26833,7 +26833,7 @@
     </row>
     <row r="372">
       <c r="A372">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B372">
         <v>32935</v>
@@ -26851,7 +26851,7 @@
     </row>
     <row r="373">
       <c r="A373">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B373">
         <v>32935</v>
@@ -26869,7 +26869,7 @@
     </row>
     <row r="374">
       <c r="A374">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B374">
         <v>32935</v>
@@ -26887,7 +26887,7 @@
     </row>
     <row r="375">
       <c r="A375">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B375">
         <v>32935</v>
@@ -26905,7 +26905,7 @@
     </row>
     <row r="376">
       <c r="A376">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B376">
         <v>32935</v>
@@ -26923,7 +26923,7 @@
     </row>
     <row r="377">
       <c r="A377">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B377">
         <v>32935</v>
@@ -26941,7 +26941,7 @@
     </row>
     <row r="378">
       <c r="A378">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B378">
         <v>32935</v>
@@ -26959,7 +26959,7 @@
     </row>
     <row r="379">
       <c r="A379">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B379">
         <v>32935</v>
@@ -26977,7 +26977,7 @@
     </row>
     <row r="380">
       <c r="A380">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B380">
         <v>32935</v>
@@ -26995,7 +26995,7 @@
     </row>
     <row r="381">
       <c r="A381">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B381">
         <v>32935</v>
@@ -27013,7 +27013,7 @@
     </row>
     <row r="382">
       <c r="A382">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B382">
         <v>32935</v>
@@ -27031,7 +27031,7 @@
     </row>
     <row r="383">
       <c r="A383">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B383">
         <v>32935</v>
@@ -27049,7 +27049,7 @@
     </row>
     <row r="384">
       <c r="A384">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B384">
         <v>32935</v>
@@ -27067,7 +27067,7 @@
     </row>
     <row r="385">
       <c r="A385">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B385">
         <v>32935</v>
@@ -27085,7 +27085,7 @@
     </row>
     <row r="386">
       <c r="A386">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B386">
         <v>32935</v>
@@ -27103,7 +27103,7 @@
     </row>
     <row r="387">
       <c r="A387">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B387">
         <v>32935</v>
@@ -27121,7 +27121,7 @@
     </row>
     <row r="388">
       <c r="A388">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B388">
         <v>32935</v>
@@ -27139,7 +27139,7 @@
     </row>
     <row r="389">
       <c r="A389">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B389">
         <v>32935</v>
@@ -27157,7 +27157,7 @@
     </row>
     <row r="390">
       <c r="A390">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B390">
         <v>32935</v>
@@ -27175,7 +27175,7 @@
     </row>
     <row r="391">
       <c r="A391">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B391">
         <v>32935</v>
@@ -27193,7 +27193,7 @@
     </row>
     <row r="392">
       <c r="A392">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B392">
         <v>32935</v>
@@ -27211,7 +27211,7 @@
     </row>
     <row r="393">
       <c r="A393">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B393">
         <v>32935</v>
@@ -27229,7 +27229,7 @@
     </row>
     <row r="394">
       <c r="A394">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B394">
         <v>32935</v>
@@ -27247,7 +27247,7 @@
     </row>
     <row r="395">
       <c r="A395">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B395">
         <v>32935</v>
@@ -27265,7 +27265,7 @@
     </row>
     <row r="396">
       <c r="A396">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B396">
         <v>32935</v>
@@ -27283,7 +27283,7 @@
     </row>
     <row r="397">
       <c r="A397">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B397">
         <v>32935</v>
@@ -27301,7 +27301,7 @@
     </row>
     <row r="398">
       <c r="A398">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B398">
         <v>32935</v>
@@ -27319,7 +27319,7 @@
     </row>
     <row r="399">
       <c r="A399">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B399">
         <v>32935</v>
@@ -27337,7 +27337,7 @@
     </row>
     <row r="400">
       <c r="A400">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B400">
         <v>32935</v>
@@ -27355,7 +27355,7 @@
     </row>
     <row r="401">
       <c r="A401">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B401">
         <v>32935</v>
@@ -27373,7 +27373,7 @@
     </row>
     <row r="402">
       <c r="A402">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B402">
         <v>32935</v>
@@ -27391,7 +27391,7 @@
     </row>
     <row r="403">
       <c r="A403">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B403">
         <v>32935</v>
@@ -27409,7 +27409,7 @@
     </row>
     <row r="404">
       <c r="A404">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B404">
         <v>32935</v>
@@ -27427,7 +27427,7 @@
     </row>
     <row r="405">
       <c r="A405">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B405">
         <v>32935</v>
@@ -27445,7 +27445,7 @@
     </row>
     <row r="406">
       <c r="A406">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B406">
         <v>32935</v>
@@ -27463,7 +27463,7 @@
     </row>
     <row r="407">
       <c r="A407">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B407">
         <v>32935</v>
@@ -27481,7 +27481,7 @@
     </row>
     <row r="408">
       <c r="A408">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B408">
         <v>32935</v>
@@ -27499,7 +27499,7 @@
     </row>
     <row r="409">
       <c r="A409">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B409">
         <v>32935</v>
@@ -27517,7 +27517,7 @@
     </row>
     <row r="410">
       <c r="A410">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B410">
         <v>32935</v>
@@ -27535,7 +27535,7 @@
     </row>
     <row r="411">
       <c r="A411">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B411">
         <v>32935</v>
@@ -27553,7 +27553,7 @@
     </row>
     <row r="412">
       <c r="A412">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B412">
         <v>32935</v>
@@ -27571,7 +27571,7 @@
     </row>
     <row r="413">
       <c r="A413">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B413">
         <v>32935</v>
@@ -27589,7 +27589,7 @@
     </row>
     <row r="414">
       <c r="A414">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B414">
         <v>32935</v>
@@ -27607,7 +27607,7 @@
     </row>
     <row r="415">
       <c r="A415">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B415">
         <v>32935</v>
@@ -27625,7 +27625,7 @@
     </row>
     <row r="416">
       <c r="A416">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B416">
         <v>32935</v>
@@ -27643,7 +27643,7 @@
     </row>
     <row r="417">
       <c r="A417">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B417">
         <v>32935</v>
@@ -27661,7 +27661,7 @@
     </row>
     <row r="418">
       <c r="A418">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B418">
         <v>32935</v>
@@ -27679,7 +27679,7 @@
     </row>
     <row r="419">
       <c r="A419">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B419">
         <v>32935</v>
@@ -27697,7 +27697,7 @@
     </row>
     <row r="420">
       <c r="A420">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B420">
         <v>32935</v>
@@ -27715,7 +27715,7 @@
     </row>
     <row r="421">
       <c r="A421">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B421">
         <v>32935</v>
@@ -27733,7 +27733,7 @@
     </row>
     <row r="422">
       <c r="A422">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B422">
         <v>32935</v>
@@ -27751,7 +27751,7 @@
     </row>
     <row r="423">
       <c r="A423">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B423">
         <v>32935</v>
@@ -27769,7 +27769,7 @@
     </row>
     <row r="424">
       <c r="A424">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B424">
         <v>32935</v>
@@ -27787,7 +27787,7 @@
     </row>
     <row r="425">
       <c r="A425">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B425">
         <v>32935</v>
@@ -27805,7 +27805,7 @@
     </row>
     <row r="426">
       <c r="A426">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B426">
         <v>32935</v>
@@ -27823,7 +27823,7 @@
     </row>
     <row r="427">
       <c r="A427">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B427">
         <v>32935</v>
@@ -27841,7 +27841,7 @@
     </row>
     <row r="428">
       <c r="A428">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B428">
         <v>32935</v>
@@ -27859,7 +27859,7 @@
     </row>
     <row r="429">
       <c r="A429">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B429">
         <v>32935</v>
@@ -27877,7 +27877,7 @@
     </row>
     <row r="430">
       <c r="A430">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B430">
         <v>32935</v>
@@ -27895,7 +27895,7 @@
     </row>
     <row r="431">
       <c r="A431">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B431">
         <v>32935</v>
@@ -27913,7 +27913,7 @@
     </row>
     <row r="432">
       <c r="A432">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B432">
         <v>32935</v>
@@ -27931,7 +27931,7 @@
     </row>
     <row r="433">
       <c r="A433">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B433">
         <v>32935</v>
@@ -27949,7 +27949,7 @@
     </row>
     <row r="434">
       <c r="A434">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B434">
         <v>32935</v>

</xml_diff>